<commit_message>
feat: redesign homepage and listing pages, add legal pages
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/intern-part2/Business-Listing/frontend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{819DD25D-E7A7-44C0-9756-3B1AAACB2D1C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="37">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -113,6 +113,24 @@
   </si>
   <si>
     <t>chore: complete initial project setup, sitemap and wireframes</t>
+  </si>
+  <si>
+    <t>Day 2</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Created the Listing Page wireframe and participated in project meetings to discuss requirements, overall direction, and design decisions. Discussed the project with the backend developer, including design suggestions and technical considerations. Researched AutoHub and similar automotive listing websites to understand common layouts and design patterns. Redesigned the mobile and desktop versions of the Homepage and Listing Page based on the research and project discussions. Created the Terms &amp; Conditions and Privacy Policy pages, added them to the sitemap, and implemented the initial boilerplate structure for both pages.Continued designing the remaining wireframes to establish the overall structure and user flow of the website.</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>feat: redesign for  homepage and listing pages, add terms and privacy pages</t>
+  </si>
+  <si>
+    <t>Waiting for new Wireframe approvals.</t>
   </si>
 </sst>
 </file>
@@ -640,7 +658,7 @@
         <v>28</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="F6" s="2">
         <v>8</v>
@@ -652,19 +670,29 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="198" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="3"/>
+      <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="F7" s="2">
+        <v>8</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">

</xml_diff>

<commit_message>
feat: add listing details and business registration wireframes
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/intern-part2/Business-Listing/frontend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/New folder/Business-Listing/frontend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{819DD25D-E7A7-44C0-9756-3B1AAACB2D1C}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4918C2F2-D422-4B9E-BC1C-6E1DB8967523}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="41">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -131,6 +131,18 @@
   </si>
   <si>
     <t>Waiting for new Wireframe approvals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day 3 </t>
+  </si>
+  <si>
+    <t>Today, I researched existing automotive listing platforms to gather design and layout ideas before creating the Listing Details Page wireframes for both mobile and desktop versions. I designed a total of 8 wireframes, including the Listing Details Page and five pages for the Business Registration Form, using a new design approach based on the research conducted. I also had a meeting with the backend developer to discuss ideas, review the project requirements, receive feedback and approval on the newer designs, and check the progress of the backend development to ensure the frontend designs remained aligned with the overall project direction.</t>
+  </si>
+  <si>
+    <t>feat: add listing details and business registration wireframes</t>
+  </si>
+  <si>
+    <t>Designs were reviewed with the backend developer and adjusted based on feedback.</t>
   </si>
 </sst>
 </file>
@@ -217,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -234,6 +246,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -694,19 +709,29 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4</v>
       </c>
       <c r="B8" s="3"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="3"/>
+      <c r="C8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="F8" s="2">
+        <v>8</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2">

</xml_diff>

<commit_message>
feat: complete frontend wireframes and project sitemap
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/New folder/Business-Listing/frontend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/Intern part 3/Business-Listing/frontend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4918C2F2-D422-4B9E-BC1C-6E1DB8967523}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78C18681-2E37-4D4A-A7EE-2D980D8B77F0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="45">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -143,13 +143,25 @@
   </si>
   <si>
     <t>Designs were reviewed with the backend developer and adjusted based on feedback.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day 4 </t>
+  </si>
+  <si>
+    <t>Completed the remaining frontend wireframes and finalized the overall wireframe design process after completing the necessary research for the frontend. Created 9 additional wireframes, bringing the total to 36 wireframes across both mobile and desktop versions. Finalized the page structures, layouts, and user flows to establish a complete foundation for frontend development. Discussed the overall page layout and design structure with the backend developer to ensure alignment between the frontend and backend implementation. Also created and completed the full project sitemap, organizing all pages and their relationships within the website.</t>
+  </si>
+  <si>
+    <t>feat: complete frontend wireframes and project sitemap</t>
+  </si>
+  <si>
+    <t>Wireframes and sitemap completed successfully. Layout and design decisions were discussed with the backend developer to ensure alignment with the project requirements and development direction.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +192,17 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial   "/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -229,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -246,7 +269,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -581,7 +610,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -593,7 +622,7 @@
     <col min="8" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="24" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>26</v>
       </c>
@@ -605,7 +634,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="16.05" customHeight="1">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -617,7 +646,7 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="22.05" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -643,11 +672,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="26.4">
       <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="3"/>
+      <c r="B5" s="8">
+        <v>46258</v>
+      </c>
       <c r="C5" s="4" t="s">
         <v>9</v>
       </c>
@@ -661,11 +692,13 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="171.6">
       <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="8">
+        <v>46259</v>
+      </c>
       <c r="C6" s="2" t="s">
         <v>27</v>
       </c>
@@ -685,11 +718,13 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="198" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="198">
       <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="3"/>
+      <c r="B7" s="8">
+        <v>46260</v>
+      </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
       </c>
@@ -709,15 +744,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="172.2">
       <c r="A8" s="2">
         <v>4</v>
       </c>
-      <c r="B8" s="3"/>
+      <c r="B8" s="8">
+        <v>46261</v>
+      </c>
       <c r="C8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -733,21 +770,33 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="172.2">
       <c r="A9" s="2">
         <v>5</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
+      <c r="B9" s="8">
+        <v>46262</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>42</v>
+      </c>
       <c r="E9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="F9" s="2">
+        <v>8</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -765,7 +814,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -779,7 +828,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -793,7 +842,7 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -807,7 +856,7 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -821,7 +870,7 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -839,7 +888,7 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -853,7 +902,7 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -867,7 +916,7 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -881,7 +930,7 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8">
       <c r="A19" s="2">
         <v>15</v>
       </c>
@@ -895,7 +944,7 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="26.4">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -913,7 +962,7 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8">
       <c r="A21" s="2">
         <v>17</v>
       </c>
@@ -927,7 +976,7 @@
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8">
       <c r="A22" s="2">
         <v>18</v>
       </c>
@@ -941,7 +990,7 @@
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8">
       <c r="A23" s="2">
         <v>19</v>
       </c>
@@ -955,7 +1004,7 @@
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8">
       <c r="A24" s="2">
         <v>20</v>
       </c>
@@ -969,7 +1018,7 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8">
       <c r="A25" s="2">
         <v>21</v>
       </c>
@@ -987,7 +1036,7 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8">
       <c r="A26" s="2">
         <v>22</v>
       </c>
@@ -1001,7 +1050,7 @@
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8">
       <c r="A27" s="2">
         <v>23</v>
       </c>
@@ -1015,7 +1064,7 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8">
       <c r="A28" s="2">
         <v>24</v>
       </c>
@@ -1029,7 +1078,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8">
       <c r="A29" s="2">
         <v>25</v>
       </c>
@@ -1043,7 +1092,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8">
       <c r="A30" s="2">
         <v>26</v>
       </c>
@@ -1061,7 +1110,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8">
       <c r="A31" s="2">
         <v>27</v>
       </c>
@@ -1075,7 +1124,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8">
       <c r="A32" s="2">
         <v>28</v>
       </c>
@@ -1089,7 +1138,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8">
       <c r="A33" s="2">
         <v>29</v>
       </c>
@@ -1103,7 +1152,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8">
       <c r="A34" s="2">
         <v>30</v>
       </c>
@@ -1117,7 +1166,7 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8">
       <c r="A35" s="2">
         <v>31</v>
       </c>
@@ -1135,7 +1184,7 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8">
       <c r="A36" s="2">
         <v>32</v>
       </c>
@@ -1149,7 +1198,7 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8">
       <c r="A37" s="2">
         <v>33</v>
       </c>
@@ -1163,7 +1212,7 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8">
       <c r="A38" s="2">
         <v>34</v>
       </c>
@@ -1177,7 +1226,7 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8">
       <c r="A39" s="2">
         <v>35</v>
       </c>
@@ -1191,7 +1240,7 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
     </row>
-    <row r="40" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="26.4">
       <c r="A40" s="2">
         <v>36</v>
       </c>
@@ -1209,7 +1258,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8">
       <c r="A41" s="2">
         <v>37</v>
       </c>
@@ -1223,7 +1272,7 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8">
       <c r="A42" s="2">
         <v>38</v>
       </c>
@@ -1237,7 +1286,7 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8">
       <c r="A43" s="2">
         <v>39</v>
       </c>
@@ -1251,7 +1300,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8">
       <c r="A44" s="2">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
fix: adjust mobile wireframes for responsive sizing
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/833f3e806b4a402c/Desktop/Intern part 3/Business-Listing/frontend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78C18681-2E37-4D4A-A7EE-2D980D8B77F0}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{7C3ED9B4-7D7E-412D-9579-AEF27658C89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DDEFACB-A74D-46BC-A050-1498834CB291}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="49">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -155,6 +155,18 @@
   </si>
   <si>
     <t>Wireframes and sitemap completed successfully. Layout and design decisions were discussed with the backend developer to ensure alignment with the project requirements and development direction.</t>
+  </si>
+  <si>
+    <t>Day 5</t>
+  </si>
+  <si>
+    <t>fix: adjust mobile wireframes for responsive sizing</t>
+  </si>
+  <si>
+    <t>Finalized the remaining wireframe adjustments and completed preparation for the frontend development phase. Researched the upcoming tasks and requirements to ensure readiness for next week.</t>
+  </si>
+  <si>
+    <t>Conducted research on frontend coding implementation and explored how the completed wireframes could be translated into code. Researched coding techniques, component implementation, and development approaches for the upcoming frontend development phase. Reviewed and revised several mobile wireframes to resolve sizing and responsive design issues. Researched and reviewed the tasks and requirements planned for the following week. Updated the Trello board with completed tasks and upcoming work, completing the planned activities for Week 1.</t>
   </si>
 </sst>
 </file>
@@ -266,9 +278,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -278,6 +287,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -322,6 +334,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -609,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -623,28 +639,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="4" spans="1:8" ht="22.05" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -674,9 +690,9 @@
     </row>
     <row r="5" spans="1:8" ht="26.4">
       <c r="A5" s="2">
-        <v>1</v>
-      </c>
-      <c r="B5" s="8">
+        <v>0</v>
+      </c>
+      <c r="B5" s="5">
         <v>46258</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -694,9 +710,9 @@
     </row>
     <row r="6" spans="1:8" ht="171.6">
       <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="8">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5">
         <v>46259</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -720,9 +736,9 @@
     </row>
     <row r="7" spans="1:8" ht="198">
       <c r="A7" s="2">
-        <v>3</v>
-      </c>
-      <c r="B7" s="8">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5">
         <v>46260</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -746,15 +762,15 @@
     </row>
     <row r="8" spans="1:8" ht="172.2">
       <c r="A8" s="2">
-        <v>4</v>
-      </c>
-      <c r="B8" s="8">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5">
         <v>46261</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="6" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -772,15 +788,15 @@
     </row>
     <row r="9" spans="1:8" ht="172.2">
       <c r="A9" s="2">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5">
         <v>46262</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="7" t="s">
         <v>42</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -796,31 +812,43 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" ht="159">
       <c r="A10" s="2">
-        <v>6</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46264</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="F10" s="2">
+        <v>8</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="3"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="3"/>
+      <c r="C11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
       </c>
@@ -830,7 +858,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="2"/>
@@ -844,7 +872,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="2"/>
@@ -858,7 +886,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="2"/>
@@ -872,15 +900,11 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="3"/>
       <c r="E15" s="2" t="s">
         <v>11</v>
       </c>
@@ -890,11 +914,15 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="3"/>
+      <c r="C16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="E16" s="2" t="s">
         <v>11</v>
       </c>
@@ -904,7 +932,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="2"/>
@@ -918,7 +946,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="2"/>
@@ -932,7 +960,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="2"/>
@@ -944,17 +972,13 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:8" ht="26.4">
+    <row r="20" spans="1:8">
       <c r="A20" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B20" s="3"/>
-      <c r="C20" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="3"/>
       <c r="E20" s="2" t="s">
         <v>11</v>
       </c>
@@ -962,13 +986,17 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" ht="26.4">
       <c r="A21" s="2">
+        <v>16</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="3"/>
       <c r="E21" s="2" t="s">
         <v>11</v>
       </c>
@@ -978,7 +1006,7 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="2"/>
@@ -992,7 +1020,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="2"/>
@@ -1006,7 +1034,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="2"/>
@@ -1020,15 +1048,11 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B25" s="3"/>
-      <c r="C25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="3"/>
       <c r="E25" s="2" t="s">
         <v>11</v>
       </c>
@@ -1038,11 +1062,15 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B26" s="3"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="3"/>
+      <c r="C26" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="E26" s="2" t="s">
         <v>11</v>
       </c>
@@ -1052,7 +1080,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="2"/>
@@ -1066,7 +1094,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="2"/>
@@ -1080,7 +1108,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="2"/>
@@ -1094,15 +1122,11 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="2">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" s="3"/>
-      <c r="C30" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="3"/>
       <c r="E30" s="2" t="s">
         <v>11</v>
       </c>
@@ -1112,11 +1136,15 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B31" s="3"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="3"/>
+      <c r="C31" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="E31" s="2" t="s">
         <v>11</v>
       </c>
@@ -1126,7 +1154,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="2"/>
@@ -1140,7 +1168,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="2"/>
@@ -1154,7 +1182,7 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="2"/>
@@ -1168,15 +1196,11 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B35" s="3"/>
-      <c r="C35" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>23</v>
-      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="3"/>
       <c r="E35" s="2" t="s">
         <v>11</v>
       </c>
@@ -1186,11 +1210,15 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="3"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="3"/>
+      <c r="C36" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="E36" s="2" t="s">
         <v>11</v>
       </c>
@@ -1200,7 +1228,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="2"/>
@@ -1214,7 +1242,7 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="2"/>
@@ -1228,7 +1256,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="2"/>
@@ -1240,17 +1268,13 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
     </row>
-    <row r="40" spans="1:8" ht="26.4">
+    <row r="40" spans="1:8">
       <c r="A40" s="2">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B40" s="3"/>
-      <c r="C40" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="3"/>
       <c r="E40" s="2" t="s">
         <v>11</v>
       </c>
@@ -1258,13 +1282,17 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" ht="26.4">
       <c r="A41" s="2">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B41" s="3"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="3"/>
+      <c r="C41" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="E41" s="2" t="s">
         <v>11</v>
       </c>
@@ -1274,7 +1302,7 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B42" s="3"/>
       <c r="C42" s="2"/>
@@ -1288,7 +1316,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B43" s="3"/>
       <c r="C43" s="2"/>
@@ -1302,7 +1330,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="2"/>
@@ -1313,13 +1341,27 @@
       <c r="F44" s="2"/>
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="2">
+        <v>40</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="2"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E44">
+  <conditionalFormatting sqref="E5:E45">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Todo"</formula>
     </cfRule>
@@ -1334,7 +1376,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="E5:E44" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="E5:E45" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Complete"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: finalize and optimize homepage for mobile and desktop
</commit_message>
<xml_diff>
--- a/frontend/Frontend-Daily-Tracker.xlsx
+++ b/frontend/Frontend-Daily-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\intern 2\Business-Listing\frontend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54282D4-33BF-4968-B104-6467248DA8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCC470C-3644-4394-B658-A0F311479254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="61">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>

</xml_diff>